<commit_message>
feat: date-agnostic site and workbook
Scheduling dates become relative so the material survives teaching
faster or slower: the setup session is "our next class", and the roster
is due "before you leave the setup session", each with a line pointing
at the course site for exact dates. Verification dates on product facts
are kept as provenance, since they record when a claim was checked.

Regenerates the roster workbook from its generator, and stops tracking
Office lock files.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TTKe9uczBQhzC5C15FTqQz
</commit_message>
<xml_diff>
--- a/forms/isom472-team-roster.xlsx
+++ b/forms/isom472-team-roster.xlsx
@@ -604,7 +604,7 @@
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Format: 16/09/2026</t>
+          <t>Format: DD/MM/YYYY</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1222,7 @@
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>Before you leave the setup session on Wednesday 16 September 2026.</t>
+          <t>Before you leave the setup session. Exact dates are announced in class and on the course site.</t>
         </is>
       </c>
     </row>

</xml_diff>